<commit_message>
BA Part 1: removed escalation process and communication standards from artifact 4 (AI and Manual)
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/BA/Part 1_Stakeholder Analysis amp Management-20260912/Done/AI/Artifacts/4. Communication Plan_VNS.xlsx
+++ b/BA/Part 1_Stakeholder Analysis amp Management-20260912/Done/AI/Artifacts/4. Communication Plan_VNS.xlsx
@@ -89,7 +89,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="5">
+  <borders count="6">
     <border>
       <left/>
       <right/>
@@ -136,6 +136,17 @@
       <right style="thin">
         <color rgb="00B4C6E7"/>
       </right>
+      <top style="thin">
+        <color rgb="00B4C6E7"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00B4C6E7"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
       <top style="thin">
         <color rgb="00B4C6E7"/>
       </top>
@@ -543,7 +554,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="B2:G35"/>
+  <dimension ref="A2:H60"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
@@ -573,6 +584,7 @@
           <t>Initiation</t>
         </is>
       </c>
+      <c r="D4" s="8" t="n"/>
       <c r="E4" s="2" t="inlineStr">
         <is>
           <t>Date</t>
@@ -583,6 +595,7 @@
           <t>02/10/2026</t>
         </is>
       </c>
+      <c r="G4" s="8" t="n"/>
     </row>
     <row r="5" ht="18" customHeight="1">
       <c r="B5" s="2" t="inlineStr">
@@ -595,6 +608,7 @@
           <t>Nazar Zankovych, Project Manager</t>
         </is>
       </c>
+      <c r="D5" s="8" t="n"/>
       <c r="E5" s="2" t="inlineStr">
         <is>
           <t>Version</t>
@@ -605,6 +619,7 @@
           <t>V1.2</t>
         </is>
       </c>
+      <c r="G5" s="8" t="n"/>
     </row>
     <row r="6" ht="18" customHeight="1">
       <c r="B6" s="2" t="inlineStr">
@@ -617,6 +632,7 @@
           <t>English for documentation; Ukrainian for day-to-day team work</t>
         </is>
       </c>
+      <c r="D6" s="8" t="n"/>
       <c r="E6" s="2" t="inlineStr">
         <is>
           <t>Validity period</t>
@@ -627,6 +643,7 @@
           <t>22/09/2026 – 31/01/2027</t>
         </is>
       </c>
+      <c r="G6" s="8" t="n"/>
     </row>
     <row r="8" ht="26" customHeight="1">
       <c r="B8" s="4" t="inlineStr">
@@ -1044,232 +1061,56 @@
         </is>
       </c>
     </row>
-    <row r="22">
-      <c r="B22" s="6" t="inlineStr">
-        <is>
-          <t>COMMUNICATION ESCALATION PROCESS</t>
-        </is>
-      </c>
-    </row>
-    <row r="23" ht="22" customHeight="1">
-      <c r="B23" s="7" t="inlineStr">
-        <is>
-          <t>Priority</t>
-        </is>
-      </c>
-      <c r="C23" s="7" t="inlineStr">
-        <is>
-          <t>Definition</t>
-        </is>
-      </c>
-      <c r="D23" s="8" t="n"/>
-      <c r="E23" s="7" t="inlineStr">
-        <is>
-          <t>Decision Authority</t>
-        </is>
-      </c>
-      <c r="F23" s="7" t="inlineStr">
-        <is>
-          <t>Timeframe for Resolution</t>
-        </is>
-      </c>
-      <c r="G23" s="8" t="n"/>
-    </row>
-    <row r="24" ht="32" customHeight="1">
-      <c r="B24" s="9" t="inlineStr">
-        <is>
-          <t>Priority 1</t>
-        </is>
-      </c>
-      <c r="C24" s="3" t="inlineStr">
-        <is>
-          <t>Major impact: the team is blocked, or the pilot or project deadline is at risk</t>
-        </is>
-      </c>
-      <c r="E24" s="3" t="inlineStr">
-        <is>
-          <t>Lviv Polytechnic National University (Sponsor)</t>
-        </is>
-      </c>
-      <c r="F24" s="3" t="inlineStr">
-        <is>
-          <t>Within 1 business day</t>
-        </is>
-      </c>
-    </row>
-    <row r="25" ht="32" customHeight="1">
-      <c r="B25" s="9" t="inlineStr">
-        <is>
-          <t>Priority 2</t>
-        </is>
-      </c>
-      <c r="C25" s="3" t="inlineStr">
-        <is>
-          <t>Medium impact: individual activities or the MVP scope may slip</t>
-        </is>
-      </c>
-      <c r="E25" s="3" t="inlineStr">
-        <is>
-          <t>Product Owner</t>
-        </is>
-      </c>
-      <c r="F25" s="3" t="inlineStr">
-        <is>
-          <t>Within 2 business days</t>
-        </is>
-      </c>
-    </row>
-    <row r="26" ht="32" customHeight="1">
-      <c r="B26" s="9" t="inlineStr">
-        <is>
-          <t>Priority 3</t>
-        </is>
-      </c>
-      <c r="C26" s="3" t="inlineStr">
-        <is>
-          <t>Slight impact: minor scheduling difficulties with no effect on scope or outcome</t>
-        </is>
-      </c>
-      <c r="E26" s="3" t="inlineStr">
-        <is>
-          <t>Project Manager</t>
-        </is>
-      </c>
-      <c r="F26" s="3" t="inlineStr">
-        <is>
-          <t>Within 3 business days</t>
-        </is>
-      </c>
-    </row>
-    <row r="27" ht="32" customHeight="1">
-      <c r="B27" s="9" t="inlineStr">
-        <is>
-          <t>Priority 4</t>
-        </is>
-      </c>
-      <c r="C27" s="3" t="inlineStr">
-        <is>
-          <t>No impact on the project, but a better solution may exist</t>
-        </is>
-      </c>
-      <c r="E27" s="3" t="inlineStr">
-        <is>
-          <t>Project Manager</t>
-        </is>
-      </c>
-      <c r="F27" s="3" t="inlineStr">
-        <is>
-          <t>Handled through the change management process</t>
-        </is>
-      </c>
-    </row>
-    <row r="29">
-      <c r="B29" s="6" t="inlineStr">
-        <is>
-          <t>COMMUNICATION STANDARDS</t>
-        </is>
-      </c>
-    </row>
-    <row r="30" ht="30" customHeight="1">
-      <c r="B30" s="10" t="inlineStr">
-        <is>
-          <t>Meeting agenda</t>
-        </is>
-      </c>
-      <c r="C30" s="3" t="inlineStr">
-        <is>
-          <t>Distributed to participants no later than 2 business days before the meeting; identifies the topics, the presenter and a time limit for each. The first item is always a review of action items from the previous meeting.</t>
-        </is>
-      </c>
-    </row>
-    <row r="31" ht="30" customHeight="1">
-      <c r="B31" s="10" t="inlineStr">
-        <is>
-          <t>Meeting minutes</t>
-        </is>
-      </c>
-      <c r="C31" s="3" t="inlineStr">
-        <is>
-          <t>Published within 1 business day after the meeting; contain the decisions taken, new action items with a named owner and due date, and the Parking Lot list.</t>
-        </is>
-      </c>
-    </row>
-    <row r="32" ht="30" customHeight="1">
-      <c r="B32" s="10" t="inlineStr">
-        <is>
-          <t>Channels</t>
-        </is>
-      </c>
-      <c r="C32" s="3" t="inlineStr">
-        <is>
-          <t>Formal documents and approvals — university @lpnu.ua mailboxes. Day-to-day team work — team chat. Tasks and defects — issue tracker.</t>
-        </is>
-      </c>
-    </row>
-    <row r="33" ht="30" customHeight="1">
-      <c r="B33" s="10" t="inlineStr">
-        <is>
-          <t>Confidentiality</t>
-        </is>
-      </c>
-      <c r="C33" s="3" t="inlineStr">
-        <is>
-          <t>Personal data of students and lecturers is not distributed through external channels. Any transfer of course materials to the external LLM API is approved by Lviv Polytechnic National University as the owner of the data.</t>
-        </is>
-      </c>
-    </row>
-    <row r="34" ht="30" customHeight="1">
-      <c r="B34" s="10" t="inlineStr">
-        <is>
-          <t>Escalation rule</t>
-        </is>
-      </c>
-      <c r="C34" s="3" t="inlineStr">
-        <is>
-          <t>Issues involving personal data or the transfer of materials to the external LLM API are escalated to the sponsor regardless of the priority assigned.</t>
-        </is>
-      </c>
-    </row>
-    <row r="35" ht="30" customHeight="1">
-      <c r="B35" s="10" t="inlineStr">
-        <is>
-          <t>Link to the register</t>
-        </is>
-      </c>
-      <c r="C35" s="3" t="inlineStr">
-        <is>
-          <t>The frequency and method of each communication match the “Preferable way of communication” and “Frequency of Communication” columns in “1. Stakeholder Register_VNS.xlsx”.</t>
-        </is>
-      </c>
-    </row>
+    <row r="21"/>
+    <row r="22"/>
+    <row r="23"/>
+    <row r="24"/>
+    <row r="25"/>
+    <row r="26"/>
+    <row r="27"/>
+    <row r="28"/>
+    <row r="29"/>
+    <row r="30"/>
+    <row r="31"/>
+    <row r="32"/>
+    <row r="33"/>
+    <row r="34"/>
+    <row r="35"/>
+    <row r="36"/>
+    <row r="37"/>
+    <row r="38"/>
+    <row r="39"/>
+    <row r="40"/>
+    <row r="41"/>
+    <row r="42"/>
+    <row r="43"/>
+    <row r="44"/>
+    <row r="45"/>
+    <row r="46"/>
+    <row r="47"/>
+    <row r="48"/>
+    <row r="49"/>
+    <row r="50"/>
+    <row r="51"/>
+    <row r="52"/>
+    <row r="53"/>
+    <row r="54"/>
+    <row r="55"/>
+    <row r="56"/>
+    <row r="57"/>
+    <row r="58"/>
+    <row r="59"/>
+    <row r="60"/>
   </sheetData>
   <autoFilter ref="B8:G20"/>
-  <mergeCells count="25">
+  <mergeCells count="7">
     <mergeCell ref="B2:G2"/>
     <mergeCell ref="F4:G4"/>
-    <mergeCell ref="C30:G30"/>
     <mergeCell ref="C6:D6"/>
-    <mergeCell ref="C24:D24"/>
-    <mergeCell ref="C34:G34"/>
-    <mergeCell ref="F25:G25"/>
     <mergeCell ref="C5:D5"/>
-    <mergeCell ref="C33:G33"/>
     <mergeCell ref="F6:G6"/>
-    <mergeCell ref="C26:D26"/>
-    <mergeCell ref="B29:G29"/>
     <mergeCell ref="C4:D4"/>
-    <mergeCell ref="C35:G35"/>
-    <mergeCell ref="F24:G24"/>
-    <mergeCell ref="C25:D25"/>
     <mergeCell ref="F5:G5"/>
-    <mergeCell ref="C31:G31"/>
-    <mergeCell ref="F26:G26"/>
-    <mergeCell ref="C27:D27"/>
-    <mergeCell ref="F23:G23"/>
-    <mergeCell ref="F27:G27"/>
-    <mergeCell ref="C23:D23"/>
-    <mergeCell ref="B22:G22"/>
-    <mergeCell ref="C32:G32"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" fitToWidth="1"/>

</xml_diff>